<commit_message>
minor additions, including SimpleIsothermalVolume and new tests
</commit_message>
<xml_diff>
--- a/solution.xlsx
+++ b/solution.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D53"/>
+  <dimension ref="A1:D65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,7 +453,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Fuel Tank</t>
+          <t>Oxygen Source Tank</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -467,273 +467,273 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3447378.646584</v>
+        <v>6894757.293168</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Fuel Tank</t>
+          <t>Manifold 1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PressureNode</t>
+          <t>SimpleIncompressibleVolume</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pressure</t>
+          <t>p</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3792116.5112424</v>
+        <v>3498041.146584</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Fuel Runline</t>
+          <t>Manifold 1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>SimpleIncompressibleVolume</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>upstream_pressure</t>
+          <t>rho</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3447378.646584</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Fuel Runline</t>
+          <t>Manifold 1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>SimpleIncompressibleVolume</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>downstream_pressure</t>
+          <t>V</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2758114.658524753</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fuel Runline</t>
+          <t>Manifold 1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>SimpleIncompressibleVolume</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>density</t>
+          <t>mdot_in</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>800</v>
+        <v>8.660224738225603</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fuel Runline</t>
+          <t>Manifold 1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>SimpleIncompressibleVolume</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>mass_flow</t>
+          <t>mdot_out</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.660438481918854</v>
+        <v>8.660224738225605</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Fuel Runline</t>
+          <t>Manifold 2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>SimpleIncompressibleVolume</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Cd</t>
+          <t>p</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>4428512.878340993</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Fuel Runline</t>
+          <t>Manifold 2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>SimpleIncompressibleVolume</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>rho</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>5e-05</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ox Runline</t>
+          <t>Manifold 2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>SimpleIncompressibleVolume</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>upstream_pressure</t>
+          <t>V</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3792116.5112424</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ox Runline</t>
+          <t>Manifold 2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>SimpleIncompressibleVolume</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>downstream_pressure</t>
+          <t>mdot_in</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2218208.055326434</v>
+        <v>7.379341209036231</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Ox Runline</t>
+          <t>Manifold 2</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>SimpleIncompressibleVolume</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>density</t>
+          <t>mdot_out</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1104</v>
+        <v>7.379341320710987</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ox Runline</t>
+          <t>Manifold 3</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>SimpleIncompressibleVolume</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>mass_flow</t>
+          <t>p</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2.947537052634985</v>
+        <v>5482962.889459851</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Ox Runline</t>
+          <t>Manifold 3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>SimpleIncompressibleVolume</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Cd</t>
+          <t>rho</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Ox Runline</t>
+          <t>Manifold 3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>SimpleIncompressibleVolume</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>V</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>5e-05</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Fuel Injector Manifold</t>
+          <t>Manifold 3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -743,17 +743,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>p</t>
+          <t>mdot_in</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2758114.658524753</v>
+        <v>7.816517386304262</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Fuel Injector Manifold</t>
+          <t>Manifold 3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -763,17 +763,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>rho</t>
+          <t>mdot_out</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>800</v>
+        <v>7.816521290451564</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Fuel Injector Manifold</t>
+          <t>Mixing Manifold</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -783,17 +783,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>p</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.1287</v>
+        <v>2715843.093985097</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Fuel Injector Manifold</t>
+          <t>Mixing Manifold</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -803,17 +803,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>mdot_in</t>
+          <t>rho</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1.660438481918854</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Fuel Injector Manifold</t>
+          <t>Mixing Manifold</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -823,17 +823,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>mdot_out</t>
+          <t>V</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1.660948488754966</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ox Injector Manifold</t>
+          <t>Mixing Manifold</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -843,17 +843,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>p</t>
+          <t>mdot_in</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2218208.055326434</v>
+        <v>15.19586261116255</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ox Injector Manifold</t>
+          <t>Mixing Manifold</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -863,77 +863,77 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>rho</t>
+          <t>mdot_out</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1104</v>
+        <v>15.1958625309906</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ox Injector Manifold</t>
+          <t>Atmosphere</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SimpleIncompressibleVolume</t>
+          <t>PressureNode</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>pressure</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.1287</v>
+        <v>101325</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ox Injector Manifold</t>
+          <t>Inlet 1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SimpleIncompressibleVolume</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>mdot_in</t>
+          <t>upstream_pressure</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>2.947537052634985</v>
+        <v>6894757.293168</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Ox Injector Manifold</t>
+          <t>Inlet 1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SimpleIncompressibleVolume</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>mdot_out</t>
+          <t>downstream_pressure</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>2.952765356074709</v>
+        <v>3498041.146584</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Fuel Injector</t>
+          <t>Inlet 1</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -943,17 +943,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>upstream_pressure</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>2758114.658524753</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Fuel Injector</t>
+          <t>Inlet 1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -963,17 +963,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>downstream_pressure</t>
+          <t>mass_flow</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2068427.187950402</v>
+        <v>8.660224738225603</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Fuel Injector</t>
+          <t>Inlet 1</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -983,17 +983,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>density</t>
+          <t>Cd</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>800</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Fuel Injector</t>
+          <t>Inlet 1</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1003,17 +1003,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>mass_flow</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1.660948488754966</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Fuel Injector</t>
+          <t>Inlet 2</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1023,17 +1023,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Cd</t>
+          <t>upstream_pressure</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>6894757.293168</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Fuel Injector</t>
+          <t>Inlet 2</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1043,17 +1043,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>downstream_pressure</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>5e-05</v>
+        <v>4428512.878340993</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Ox Injector</t>
+          <t>Inlet 2</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1063,17 +1063,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>upstream_pressure</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2218208.055326434</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Ox Injector</t>
+          <t>Inlet 2</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1083,17 +1083,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>downstream_pressure</t>
+          <t>mass_flow</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>2068427.187950402</v>
+        <v>7.379341209036231</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ox Injector</t>
+          <t>Inlet 2</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1103,17 +1103,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>density</t>
+          <t>Cd</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1104</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Ox Injector</t>
+          <t>Inlet 2</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1123,17 +1123,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>mass_flow</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>2.952765356074709</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Ox Injector</t>
+          <t>Inlet 3</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1143,17 +1143,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Cd</t>
+          <t>upstream_pressure</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1</v>
+        <v>6894757.293168</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Ox Injector</t>
+          <t>Inlet 3</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1163,335 +1163,571 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>downstream_pressure</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.0001623682955088642</v>
+        <v>5482962.889459851</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Combustion Chamber</t>
+          <t>Inlet 3</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>RocketCEACombustionChamber</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>2068427.187950402</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Combustion Chamber</t>
+          <t>Inlet 3</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>RocketCEACombustionChamber</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ox_mdot</t>
+          <t>mass_flow</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>2.952765356074709</v>
+        <v>7.816517386304262</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Combustion Chamber</t>
+          <t>Inlet 3</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>RocketCEACombustionChamber</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>fuel_mdot</t>
+          <t>Cd</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>1.660948488754966</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Combustion Chamber</t>
+          <t>Inlet 3</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>RocketCEACombustionChamber</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>nozzle_mdot</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>4.617514619961214</v>
+        <v>0.00014</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Nozzle</t>
+          <t>Outlet 1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>RocketCEAChokedNozzle</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>fuel</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>RP-1</t>
-        </is>
+          <t>upstream_pressure</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>3498041.146584</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Nozzle</t>
+          <t>Outlet 1</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>RocketCEAChokedNozzle</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ox</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>LOX</t>
-        </is>
+          <t>downstream_pressure</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>101325</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Nozzle</t>
+          <t>Outlet 1</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>RocketCEAChokedNozzle</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>2068427.187950402</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Nozzle</t>
+          <t>Outlet 1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>RocketCEAChokedNozzle</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>MR</t>
+          <t>mass_flow</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1.777758537405382</v>
+        <v>8.660224738225605</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Nozzle</t>
+          <t>Outlet 1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>RocketCEAChokedNozzle</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>At</t>
+          <t>Cd</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.003903225806451613</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Nozzle</t>
+          <t>Outlet 1</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>RocketCEAChokedNozzle</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>eps</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>4</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Nozzle</t>
+          <t>Outlet 2</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>RocketCEAChokedNozzle</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Pamb</t>
+          <t>upstream_pressure</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>101325</v>
+        <v>4428512.878340993</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Nozzle</t>
+          <t>Outlet 2</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>RocketCEAChokedNozzle</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>downstream_pressure</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>889.6442958225161</v>
+        <v>2715843.093985097</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Nozzle</t>
+          <t>Outlet 2</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>RocketCEAChokedNozzle</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>mdot</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>4.617514619961214</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Nozzle</t>
+          <t>Outlet 2</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>RocketCEAChokedNozzle</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>eta_cstar</t>
+          <t>mass_flow</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>1</v>
+        <v>7.379341320710987</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Nozzle</t>
+          <t>Outlet 2</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>RocketCEAChokedNozzle</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>eta_Cf</t>
+          <t>Cd</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.0787236957286275</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Atmosphere</t>
+          <t>Outlet 2</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PressureNode</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>pressure</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D53" t="n">
+        <v>0.00012</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Outlet 3</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>upstream_pressure</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>5482962.889459851</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Outlet 3</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>downstream_pressure</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>2715843.093985097</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Outlet 3</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>density</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>1104</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Outlet 3</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>mass_flow</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>7.816521290451564</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Outlet 3</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Cd</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Outlet 3</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Drain Line</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>upstream_pressure</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>2715843.093985097</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Drain Line</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>downstream_pressure</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
         <v>101325</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Drain Line</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>density</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>1104</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Drain Line</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>mass_flow</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>15.1958625309906</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Drain Line</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Cd</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Drain Line</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>0.0002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Made fluids into generic fluid components
</commit_message>
<xml_diff>
--- a/solution.xlsx
+++ b/solution.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,12 +453,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Source Fluid</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>IsothermalPressureBoundary</t>
+          <t>DensityfromPT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -468,19 +468,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>RP-1</t>
+          <t>Water</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Source Fluid</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>IsothermalPressureBoundary</t>
+          <t>DensityfromPT</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -495,442 +495,562 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Source Fluid</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>IsothermalPressureBoundary</t>
+          <t>DensityfromPT</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>rho</t>
+          <t>temperature</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>744.5107206142487</v>
+        <v>300</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Source Fluid</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>IsothermalPressureBoundary</t>
+          <t>DensityfromPT</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>temperature</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>300</v>
+        <v>996.6461141257844</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Line 1</t>
+          <t>Manifold Fluid</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>DensityfromPT</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>upstream_pressure</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>300000</v>
+          <t>fluid</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Line 1</t>
+          <t>Manifold Fluid</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>DensityfromPT</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>downstream_pressure</t>
+          <t>pressure</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>199999.99998</v>
+        <v>200663.6036776134</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Line 1</t>
+          <t>Manifold Fluid</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>DensityfromPT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>density</t>
+          <t>temperature</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>744.4732644898204</v>
+        <v>300</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Line 1</t>
+          <t>Manifold Fluid</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>DensityfromPT</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>mass_flow</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.6101119834250096</v>
+        <v>996.6015298873724</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Line 1</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>IsothermalPressureBoundary</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Cd</t>
+          <t>pressure</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Line 1</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>IsothermalPressureBoundary</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>5e-05</v>
+        <v>996.6461141257844</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IsothermalIncompressibleVolume</t>
+          <t>IsothermalPressureBoundary</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>fluid</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>RP-1</t>
-        </is>
+          <t>temperature</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IsothermalIncompressibleVolume</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>p</t>
+          <t>upstream_pressure</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>199999.99998</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IsothermalIncompressibleVolume</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>downstream_pressure</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>300</v>
+        <v>200663.6036776134</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IsothermalIncompressibleVolume</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>rho</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>744.4358083653919</v>
+        <v>996.6238220065784</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>IsothermalIncompressibleVolume</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>mass_flow</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.02</v>
+        <v>0.7035659847063997</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>IsothermalIncompressibleVolume</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>mdot_in</t>
+          <t>Cd</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.6101119834250096</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>IsothermalIncompressibleVolume</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>mdot_out</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.6060412666459536</v>
+        <v>5e-05</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Line 2</t>
+          <t>Manifold</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>IsothermalIncompressibleVolume</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>upstream_pressure</t>
+          <t>p</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>199999.99998</v>
+        <v>200663.6036776134</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Line 2</t>
+          <t>Manifold</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>IsothermalIncompressibleVolume</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>downstream_pressure</t>
+          <t>T</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>101325</v>
+        <v>300</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Line 2</t>
+          <t>Manifold</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>IsothermalIncompressibleVolume</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>density</t>
+          <t>rho</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>744.4358083653919</v>
+        <v>996.6015298873724</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Line 2</t>
+          <t>Manifold</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>IsothermalIncompressibleVolume</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>mass_flow</t>
+          <t>V</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.6060412666459536</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Line 2</t>
+          <t>Manifold</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>IsothermalIncompressibleVolume</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Cd</t>
+          <t>mdot_in</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>0.7035659847063997</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Line 2</t>
+          <t>Manifold</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>IsothermalIncompressibleVolume</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>mdot_out</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>5e-05</v>
+        <v>0.7035659329515068</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Atmosphere</t>
+          <t>Line 2</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>upstream_pressure</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>200663.6036776134</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>downstream_pressure</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>101325</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>density</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>996.6015298873724</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>mass_flow</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>0.7035659329515068</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Cd</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>5e-05</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Atmoshere</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>PressureBoundary</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>pressure</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="D31" t="n">
         <v>101325</v>
       </c>
     </row>

</xml_diff>

<commit_message>
external States can be passed into fluid lookup component
</commit_message>
<xml_diff>
--- a/solution.xlsx
+++ b/solution.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>jeta</t>
+          <t>tone</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>300000</v>
+        <v>137895.14586336</v>
       </c>
     </row>
     <row r="4">
@@ -530,7 +530,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>jeta</t>
+          <t>tone</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>200664.975160748</v>
+        <v>119520.5129985313</v>
       </c>
     </row>
     <row r="7">
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>300000</v>
+        <v>137895.14586336</v>
       </c>
     </row>
     <row r="9">
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>744.5107206142487</v>
+        <v>782.6670025529312</v>
       </c>
     </row>
     <row r="10">
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>300000</v>
+        <v>137895.14586336</v>
       </c>
     </row>
     <row r="12">
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>200664.975160748</v>
+        <v>119520.5129985313</v>
       </c>
     </row>
     <row r="13">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>744.4735136942427</v>
+        <v>782.6574922151821</v>
       </c>
     </row>
     <row r="14">
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.6080801549754064</v>
+        <v>0.2681514877672835</v>
       </c>
     </row>
     <row r="15">
@@ -771,7 +771,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>200664.975160748</v>
+        <v>119520.5129985313</v>
       </c>
     </row>
     <row r="18">
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>744.4363067742368</v>
+        <v>782.6479818774329</v>
       </c>
     </row>
     <row r="20">
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.6080801549754064</v>
+        <v>0.2681514877672835</v>
       </c>
     </row>
     <row r="22">
@@ -871,7 +871,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.6080801107737025</v>
+        <v>0.2681483309337115</v>
       </c>
     </row>
     <row r="23">
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>200664.975160748</v>
+        <v>119520.5129985313</v>
       </c>
     </row>
     <row r="24">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>101325</v>
+        <v>101146.0894907746</v>
       </c>
     </row>
     <row r="25">
@@ -931,7 +931,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>744.4363067742368</v>
+        <v>782.6479818774329</v>
       </c>
     </row>
     <row r="26">
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.6080801107737025</v>
+        <v>0.2681483309337115</v>
       </c>
     </row>
     <row r="27">
@@ -1011,7 +1011,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>101325</v>
+        <v>101146.0894907746</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
removed the need to predfine States, also added a static evaluate to Steady State
</commit_message>
<xml_diff>
--- a/solution.xlsx
+++ b/solution.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>tone</t>
+          <t>RP-1</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Manifold Fluid</t>
+          <t>Source Fluid</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -525,12 +525,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>fluid</t>
+          <t>property_states</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>tone</t>
+          <t>{}</t>
         </is>
       </c>
     </row>
@@ -547,11 +547,13 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pressure</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>119520.5129985313</v>
+          <t>fluid</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>RP-1</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -567,51 +569,53 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>temperature</t>
+          <t>pressure</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>300</v>
+        <v>103421.35939752</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Manifold Fluid</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>IsothermalPressureBoundary</t>
+          <t>GeneralFluidLookupfromPT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>pressure</t>
+          <t>temperature</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>137895.14586336</v>
+        <v>300</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Manifold Fluid</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>IsothermalPressureBoundary</t>
+          <t>GeneralFluidLookupfromPT</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>density</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>782.6670025529312</v>
+          <t>property_states</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -627,51 +631,51 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>temperature</t>
+          <t>pressure</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>300</v>
+        <v>137895.14586336</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Line 1</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>IsothermalPressureBoundary</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>upstream_pressure</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>137895.14586336</v>
+        <v>744.3892444235298</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Line 1</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>IsothermalPressureBoundary</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>downstream_pressure</t>
+          <t>temperature</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>119520.5129985313</v>
+        <v>300</v>
       </c>
     </row>
     <row r="13">
@@ -687,11 +691,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>density</t>
+          <t>upstream_pressure</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>782.6574922151821</v>
+        <v>137895.14586336</v>
       </c>
     </row>
     <row r="14">
@@ -707,11 +711,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>mass_flow</t>
+          <t>downstream_pressure</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.2681514877672835</v>
+        <v>103421.35939752</v>
       </c>
     </row>
     <row r="15">
@@ -727,11 +731,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Cd</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>744.3763142409618</v>
       </c>
     </row>
     <row r="16">
@@ -747,51 +751,51 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>discharge_coefficient</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>5e-05</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>IsothermalIncompressibleVolume</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>p</t>
+          <t>cross_sectional_area</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>119520.5129985313</v>
+        <v>5e-05</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>IsothermalIncompressibleVolume</t>
+          <t>DischargeCoefficient</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>mass_flow</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>300</v>
+        <v>0.3582001542948575</v>
       </c>
     </row>
     <row r="19">
@@ -807,11 +811,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>rho</t>
+          <t>pressure</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>782.6479818774329</v>
+        <v>103421.35939752</v>
       </c>
     </row>
     <row r="20">
@@ -827,11 +831,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>temperature</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.01</v>
+        <v>300</v>
       </c>
     </row>
     <row r="21">
@@ -847,11 +851,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>mdot_in</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.2681514877672835</v>
+        <v>744.363384058394</v>
       </c>
     </row>
     <row r="22">
@@ -867,51 +871,51 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>mdot_out</t>
+          <t>volume</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.2681483309337115</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Line 2</t>
+          <t>Manifold</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>IsothermalIncompressibleVolume</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>upstream_pressure</t>
+          <t>mass_flow_in</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>119520.5129985313</v>
+        <v>0.3582001542948575</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Line 2</t>
+          <t>Manifold</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>IsothermalIncompressibleVolume</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>downstream_pressure</t>
+          <t>mass_flow_out</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>101146.0894907746</v>
+        <v>0.09202248658429256</v>
       </c>
     </row>
     <row r="25">
@@ -927,11 +931,11 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>density</t>
+          <t>upstream_pressure</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>782.6479818774329</v>
+        <v>103421.35939752</v>
       </c>
     </row>
     <row r="26">
@@ -947,11 +951,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>mass_flow</t>
+          <t>downstream_pressure</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.2681483309337115</v>
+        <v>101146.0894907746</v>
       </c>
     </row>
     <row r="27">
@@ -967,11 +971,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Cd</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>744.363384058394</v>
       </c>
     </row>
     <row r="28">
@@ -987,30 +991,70 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>discharge_coefficient</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>5e-05</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>cross_sectional_area</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>5e-05</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>mass_flow</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>0.09202248658429256</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>Atmoshere</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>PressureBoundary</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>pressure</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D31" t="n">
         <v>101146.0894907746</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added circular darcy weisbach component, also added least_squares + root in SteadyState. Darcy needs some updates.
</commit_message>
<xml_diff>
--- a/solution.xlsx
+++ b/solution.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>103421.35939752</v>
+        <v>137410.1557569624</v>
       </c>
     </row>
     <row r="8">
@@ -686,7 +686,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>103421.35939752</v>
+        <v>137410.1557569624</v>
       </c>
     </row>
     <row r="15">
@@ -726,16 +726,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>density</t>
+          <t>length</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>744.3763142409618</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -746,16 +746,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>discharge_coefficient</t>
+          <t>inner_diameter</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>0.0254000508001016</v>
       </c>
     </row>
     <row r="17">
@@ -766,16 +766,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>cross_sectional_area</t>
+          <t>roughness</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5e-05</v>
+        <v>9.000000000000001e-05</v>
       </c>
     </row>
     <row r="18">
@@ -786,116 +786,118 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>mass_flow</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.3582001542948575</v>
+        <v>744.3890625495426</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>IsothermalIncompressibleVolume</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>pressure</t>
+          <t>dynamic_viscosity</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>103421.35939752</v>
+        <v>0.001315977714550519</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>IsothermalIncompressibleVolume</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>temperature</t>
+          <t>Reynolds_number_threshold</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>300</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>IsothermalIncompressibleVolume</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>density</t>
+          <t>mass_flow</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>744.363384058394</v>
+        <v>0.372910750890164</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>IsothermalIncompressibleVolume</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>volume</t>
+          <t>friction_factor</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.01</v>
+        <v>0.03386146461875016</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>IsothermalIncompressibleVolume</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>mass_flow_in</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>0.3582001542948575</v>
+          <t>flow_regime</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>turbulent</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -911,111 +913,111 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>mass_flow_out</t>
+          <t>pressure</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.09202248658429256</v>
+        <v>137410.1557569624</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Line 2</t>
+          <t>Manifold</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>IsothermalIncompressibleVolume</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>upstream_pressure</t>
+          <t>temperature</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>103421.35939752</v>
+        <v>300</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Line 2</t>
+          <t>Manifold</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>IsothermalIncompressibleVolume</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>downstream_pressure</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>101146.0894907746</v>
+        <v>744.3888806755554</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Line 2</t>
+          <t>Manifold</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>IsothermalIncompressibleVolume</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>density</t>
+          <t>volume</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>744.363384058394</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Line 2</t>
+          <t>Manifold</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>IsothermalIncompressibleVolume</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>discharge_coefficient</t>
+          <t>mass_flow_in</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>0.372910750890164</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Line 2</t>
+          <t>Manifold</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>IsothermalIncompressibleVolume</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>cross_sectional_area</t>
+          <t>mass_flow_out</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>5e-05</v>
+        <v>0.367386497415404</v>
       </c>
     </row>
     <row r="30">
@@ -1031,30 +1033,130 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>mass_flow</t>
+          <t>upstream_pressure</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.09202248658429256</v>
+        <v>137410.1557569624</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>downstream_pressure</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>101146.0894907746</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>density</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>744.3888806755554</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>discharge_coefficient</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>cross_sectional_area</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>5e-05</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>DischargeCoefficient</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>mass_flow</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>0.367386497415404</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>Atmoshere</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>PressureBoundary</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>pressure</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D36" t="n">
         <v>101146.0894907746</v>
       </c>
     </row>

</xml_diff>

<commit_message>
darcy with fixed-point iteration and numerical stability wrightomega added
</commit_message>
<xml_diff>
--- a/solution.xlsx
+++ b/solution.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>RP-1</t>
+          <t>lox</t>
         </is>
       </c>
     </row>
@@ -509,13 +509,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Source Fluid</t>
+          <t>Manifold Fluid</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -525,12 +525,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>property_states</t>
+          <t>fluid</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>lox</t>
         </is>
       </c>
     </row>
@@ -547,13 +547,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>fluid</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>RP-1</t>
-        </is>
+          <t>pressure</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>133105.4452704541</v>
       </c>
     </row>
     <row r="7">
@@ -569,53 +567,51 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pressure</t>
+          <t>temperature</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>137410.1557569624</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Manifold Fluid</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GeneralFluidLookupfromPT</t>
+          <t>IsothermalPressureBoundary</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>temperature</t>
+          <t>pressure</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>300</v>
+        <v>137895.14586336</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Manifold Fluid</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>GeneralFluidLookupfromPT</t>
+          <t>IsothermalPressureBoundary</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>property_states</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
+          <t>density</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>5.486360357935013</v>
       </c>
     </row>
     <row r="10">
@@ -631,51 +627,51 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>pressure</t>
+          <t>temperature</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>137895.14586336</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IsothermalPressureBoundary</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>density</t>
+          <t>upstream_pressure</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>744.3892444235298</v>
+        <v>137895.14586336</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IsothermalPressureBoundary</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>temperature</t>
+          <t>downstream_pressure</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>300</v>
+        <v>133105.4452704541</v>
       </c>
     </row>
     <row r="13">
@@ -691,11 +687,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>upstream_pressure</t>
+          <t>length</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>137895.14586336</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -711,11 +707,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>downstream_pressure</t>
+          <t>inner_diameter</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>137410.1557569624</v>
+        <v>0.0127000254000508</v>
       </c>
     </row>
     <row r="15">
@@ -731,11 +727,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>length</t>
+          <t>roughness</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="16">
@@ -751,11 +747,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>inner_diameter</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.0254000508001016</v>
+        <v>5.387866699875579</v>
       </c>
     </row>
     <row r="17">
@@ -771,11 +767,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>roughness</t>
+          <t>dynamic_viscosity</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>9.000000000000001e-05</v>
+        <v>7.715838935354237e-06</v>
       </c>
     </row>
     <row r="18">
@@ -791,11 +787,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>density</t>
+          <t>Reynolds_number_threshold</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>744.3890625495426</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="19">
@@ -811,11 +807,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>dynamic_viscosity</t>
+          <t>mass_flow</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.001315977714550519</v>
+        <v>0.01725414891453389</v>
       </c>
     </row>
     <row r="20">
@@ -831,11 +827,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Reynolds_number_threshold</t>
+          <t>friction_factor</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>2300</v>
+        <v>0.03533221226209587</v>
       </c>
     </row>
     <row r="21">
@@ -851,11 +847,13 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>mass_flow</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>0.372910750890164</v>
+          <t>flow_regime</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>turbulent</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -871,33 +869,31 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>friction_factor</t>
+          <t>Reynolds_number</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.03386146461875016</v>
+        <v>224189.8351765289</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Line 1</t>
+          <t>Manifold</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>IsothermalIncompressibleVolume</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>flow_regime</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>turbulent</t>
-        </is>
+          <t>pressure</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>133105.4452704541</v>
       </c>
     </row>
     <row r="24">
@@ -913,11 +909,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>pressure</t>
+          <t>temperature</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>137410.1557569624</v>
+        <v>100</v>
       </c>
     </row>
     <row r="25">
@@ -933,11 +929,11 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>temperature</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>300</v>
+        <v>5.289373041816145</v>
       </c>
     </row>
     <row r="26">
@@ -953,11 +949,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>density</t>
+          <t>volume</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>744.3888806755554</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="27">
@@ -973,11 +969,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>volume</t>
+          <t>mass_flow_in</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.01</v>
+        <v>0.01725414891453389</v>
       </c>
     </row>
     <row r="28">
@@ -993,31 +989,31 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>mass_flow_in</t>
+          <t>mass_flow_out</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.372910750890164</v>
+        <v>0.01725414891453275</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Manifold</t>
+          <t>Line 2</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>IsothermalIncompressibleVolume</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>mass_flow_out</t>
+          <t>upstream_pressure</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.367386497415404</v>
+        <v>133105.4452704541</v>
       </c>
     </row>
     <row r="30">
@@ -1028,16 +1024,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>upstream_pressure</t>
+          <t>downstream_pressure</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>137410.1557569624</v>
+        <v>101146.0894907746</v>
       </c>
     </row>
     <row r="31">
@@ -1048,16 +1044,16 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>downstream_pressure</t>
+          <t>length</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>101146.0894907746</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
@@ -1068,16 +1064,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>density</t>
+          <t>inner_diameter</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>744.3888806755554</v>
+        <v>0.01016002032004064</v>
       </c>
     </row>
     <row r="33">
@@ -1088,16 +1084,16 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>discharge_coefficient</t>
+          <t>roughness</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="34">
@@ -1108,16 +1104,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>cross_sectional_area</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5e-05</v>
+        <v>5.289373041816145</v>
       </c>
     </row>
     <row r="35">
@@ -1128,35 +1124,137 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>DischargeCoefficient</t>
+          <t>DarcyWeisbach</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>mass_flow</t>
+          <t>dynamic_viscosity</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.367386497415404</v>
+        <v>7.715355294610074e-06</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>DarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Reynolds_number_threshold</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>2300</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>DarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>mass_flow</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>0.01725414891453275</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>DarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>friction_factor</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>0.03791995169040334</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>DarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>flow_regime</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>turbulent</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>DarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Reynolds_number</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>280254.860779715</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>Atmoshere</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>PressureBoundary</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>pressure</t>
         </is>
       </c>
-      <c r="D36" t="n">
+      <c r="D41" t="n">
         <v>101146.0894907746</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated steady state to have least_squares as a backup to root()
</commit_message>
<xml_diff>
--- a/solution.xlsx
+++ b/solution.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>lox</t>
+          <t>water</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
     </row>
     <row r="5">
@@ -530,7 +530,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>lox</t>
+          <t>water</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>133105.4452704541</v>
+        <v>132947.2588499769</v>
       </c>
     </row>
     <row r="7">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
     </row>
     <row r="8">
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>5.486360357935013</v>
+        <v>996.5733532570438</v>
       </c>
     </row>
     <row r="10">
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
     </row>
     <row r="11">
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>133105.4452704541</v>
+        <v>132947.2588499769</v>
       </c>
     </row>
     <row r="13">
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>5.387866699875579</v>
+        <v>996.5722426292007</v>
       </c>
     </row>
     <row r="17">
@@ -771,7 +771,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>7.715838935354237e-06</v>
+        <v>0.0008537391772258214</v>
       </c>
     </row>
     <row r="18">
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.01725414891453389</v>
+        <v>0.2317067838975991</v>
       </c>
     </row>
     <row r="20">
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.03533221226209587</v>
+        <v>0.03743551121309351</v>
       </c>
     </row>
     <row r="21">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>224189.8351765289</v>
+        <v>27209.40638612517</v>
       </c>
     </row>
     <row r="23">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>133105.4452704541</v>
+        <v>132947.2588499769</v>
       </c>
     </row>
     <row r="24">
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
     </row>
     <row r="25">
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>5.289373041816145</v>
+        <v>996.5711320013575</v>
       </c>
     </row>
     <row r="26">
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.01725414891453389</v>
+        <v>0.2317067838975991</v>
       </c>
     </row>
     <row r="28">
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.01725414891453275</v>
+        <v>0.2317067838976202</v>
       </c>
     </row>
     <row r="29">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>133105.4452704541</v>
+        <v>132947.2588499769</v>
       </c>
     </row>
     <row r="30">
@@ -1113,7 +1113,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5.289373041816145</v>
+        <v>996.5711320013575</v>
       </c>
     </row>
     <row r="35">
@@ -1133,7 +1133,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>7.715355294610074e-06</v>
+        <v>0.0008537396247040118</v>
       </c>
     </row>
     <row r="36">
@@ -1173,7 +1173,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.01725414891453275</v>
+        <v>0.2317067838976202</v>
       </c>
     </row>
     <row r="38">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.03791995169040334</v>
+        <v>0.03942090037303891</v>
       </c>
     </row>
     <row r="39">
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>280254.860779715</v>
+        <v>34011.74015577226</v>
       </c>
     </row>
     <row r="41">

</xml_diff>

<commit_message>
non-circular and generic Darcy Weisbach added
</commit_message>
<xml_diff>
--- a/solution.xlsx
+++ b/solution.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>132947.2588499769</v>
+        <v>101163.5751201206</v>
       </c>
     </row>
     <row r="7">
@@ -642,7 +642,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>132947.2588499769</v>
+        <v>101163.5751201206</v>
       </c>
     </row>
     <row r="13">
@@ -682,7 +682,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -742,7 +742,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>996.5722426292007</v>
+        <v>996.5651080242469</v>
       </c>
     </row>
     <row r="17">
@@ -762,7 +762,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -802,7 +802,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.2317067838975991</v>
+        <v>0.6443805136601886</v>
       </c>
     </row>
     <row r="20">
@@ -822,7 +822,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.03743551121309351</v>
+        <v>0.0359329676637423</v>
       </c>
     </row>
     <row r="21">
@@ -842,7 +842,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>27209.40638612517</v>
+        <v>75669.82273263442</v>
       </c>
     </row>
     <row r="23">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>132947.2588499769</v>
+        <v>101163.5751201206</v>
       </c>
     </row>
     <row r="24">
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>996.5711320013575</v>
+        <v>996.5568627914502</v>
       </c>
     </row>
     <row r="26">
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.2317067838975991</v>
+        <v>0.6443805136601886</v>
       </c>
     </row>
     <row r="28">
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.2317067838976202</v>
+        <v>0.6443805138542278</v>
       </c>
     </row>
     <row r="29">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>EllipticalDuctDarcyWeisbach</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>132947.2588499769</v>
+        <v>101163.5751201206</v>
       </c>
     </row>
     <row r="30">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>EllipticalDuctDarcyWeisbach</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>EllipticalDuctDarcyWeisbach</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1064,16 +1064,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>EllipticalDuctDarcyWeisbach</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>inner_diameter</t>
+          <t>semi_major_axis</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.01016002032004064</v>
+        <v>0.05080010160020321</v>
       </c>
     </row>
     <row r="33">
@@ -1084,16 +1084,16 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>EllipticalDuctDarcyWeisbach</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>roughness</t>
+          <t>semi_minor_axis</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.0001</v>
+        <v>0.0254000508001016</v>
       </c>
     </row>
     <row r="34">
@@ -1104,16 +1104,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>EllipticalDuctDarcyWeisbach</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>density</t>
+          <t>roughness</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>996.5711320013575</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="35">
@@ -1124,16 +1124,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>EllipticalDuctDarcyWeisbach</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>dynamic_viscosity</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.0008537396247040118</v>
+        <v>996.5568627914502</v>
       </c>
     </row>
     <row r="36">
@@ -1144,16 +1144,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>EllipticalDuctDarcyWeisbach</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Reynolds_number_threshold</t>
+          <t>dynamic_viscosity</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>2300</v>
+        <v>0.0008537425009013317</v>
       </c>
     </row>
     <row r="37">
@@ -1164,16 +1164,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>EllipticalDuctDarcyWeisbach</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>mass_flow</t>
+          <t>Reynolds_number_threshold</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.2317067838976202</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="38">
@@ -1184,16 +1184,16 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>EllipticalDuctDarcyWeisbach</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>friction_factor</t>
+          <t>mass_flow</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.03942090037303891</v>
+        <v>0.6443805138542278</v>
       </c>
     </row>
     <row r="39">
@@ -1204,18 +1204,16 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>EllipticalDuctDarcyWeisbach</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>flow_regime</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>turbulent</t>
-        </is>
+          <t>friction_factor</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>0.03215033542759246</v>
       </c>
     </row>
     <row r="40">
@@ -1226,35 +1224,57 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>DarcyWeisbach</t>
+          <t>EllipticalDuctDarcyWeisbach</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Reynolds_number</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>34011.74015577226</v>
+          <t>flow_regime</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>turbulent</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>EllipticalDuctDarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Reynolds_number</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>12268.39912283695</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>Atmoshere</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>PressureBoundary</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>pressure</t>
         </is>
       </c>
-      <c r="D41" t="n">
+      <c r="D42" t="n">
         <v>101146.0894907746</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added a simple solver penalty, descoped residual scalars for now
</commit_message>
<xml_diff>
--- a/solution.xlsx
+++ b/solution.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Octane</t>
+          <t>Water</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>137895.14586336</v>
+        <v>133065.7866534328</v>
       </c>
     </row>
     <row r="4">
@@ -530,7 +530,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Octane</t>
+          <t>Water</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>101162.5201577866</v>
+        <v>101161.4754845989</v>
       </c>
     </row>
     <row r="7">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>300.0153620160509</v>
+        <v>300.007026375315</v>
       </c>
     </row>
     <row r="8">
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>137895.14586336</v>
+        <v>133065.7866534328</v>
       </c>
     </row>
     <row r="9">
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>697.1129783549328</v>
+        <v>996.5711852123106</v>
       </c>
     </row>
     <row r="10">
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>137895.14586336</v>
+        <v>133065.7866534328</v>
       </c>
     </row>
     <row r="12">
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>101162.5201577866</v>
+        <v>101161.4754845989</v>
       </c>
     </row>
     <row r="13">
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>697.0898815262594</v>
+        <v>996.563061299966</v>
       </c>
     </row>
     <row r="17">
@@ -771,7 +771,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.0005004654720936113</v>
+        <v>0.0008537396139834584</v>
       </c>
     </row>
     <row r="18">
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.5409795888565161</v>
+        <v>0.5999999999832152</v>
       </c>
     </row>
     <row r="20">
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.03566249300640285</v>
+        <v>0.03599849656322113</v>
       </c>
     </row>
     <row r="21">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>108370.8022541713</v>
+        <v>70458.16788226328</v>
       </c>
     </row>
     <row r="23">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>101162.5201577866</v>
+        <v>101161.4754845989</v>
       </c>
     </row>
     <row r="24">
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>300.0153620160509</v>
+        <v>300.007026375315</v>
       </c>
     </row>
     <row r="25">
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>697.0667846975862</v>
+        <v>996.5549373876212</v>
       </c>
     </row>
     <row r="26">
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.5409795888565161</v>
+        <v>0.5999999999832152</v>
       </c>
     </row>
     <row r="28">
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.5409795888534189</v>
+        <v>0.5999999989554832</v>
       </c>
     </row>
     <row r="29">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>-240286.6900943597</v>
+        <v>112684.1239456321</v>
       </c>
     </row>
     <row r="30">
@@ -1033,7 +1033,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>-240286.6901602884</v>
+        <v>112684.1238040962</v>
       </c>
     </row>
     <row r="31">
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>101162.5201577866</v>
+        <v>101161.4754845989</v>
       </c>
     </row>
     <row r="32">
@@ -1173,7 +1173,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>697.0667846975862</v>
+        <v>996.5549373876212</v>
       </c>
     </row>
     <row r="38">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.0005001785853022154</v>
+        <v>0.0008536092843270284</v>
       </c>
     </row>
     <row r="39">
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.5409795888534189</v>
+        <v>0.5999999989554832</v>
       </c>
     </row>
     <row r="41">
@@ -1253,7 +1253,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.02998159807679982</v>
+        <v>0.03262956268924404</v>
       </c>
     </row>
     <row r="42">
@@ -1295,7 +1295,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>17580.37704116755</v>
+        <v>11425.21861901881</v>
       </c>
     </row>
     <row r="44">

</xml_diff>

<commit_message>
Updated Fluid and IdealGas lookups
</commit_message>
<xml_diff>
--- a/solution.xlsx
+++ b/solution.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,12 +453,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Supply Gas</t>
+          <t>Source Fluid</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>GeneralFluidLookupfromPT</t>
+          <t>FluidLookup</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -468,19 +468,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Nitrogen</t>
+          <t>Octane</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Supply Gas</t>
+          <t>Source Fluid</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>GeneralFluidLookupfromPT</t>
+          <t>FluidLookup</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -489,369 +489,833 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>20684271.879504</v>
+        <v>146271.5950004372</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Supply Gas</t>
+          <t>Source Fluid</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>GeneralFluidLookupfromPT</t>
+          <t>FluidLookup</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>temperature</t>
+          <t>enthalpy</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>300</v>
+        <v>-240286.6900943597</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Supply Gas Specific Heat</t>
+          <t>Manifold Fluid</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>IdealGasSpecificHeats</t>
+          <t>FluidLookup</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>molar_mass</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>0.02801348</v>
+          <t>fluid</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Octane</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Supply Gas Specific Heat</t>
+          <t>Manifold Fluid</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>IdealGasSpecificHeats</t>
+          <t>FluidLookup</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>degrees_of_freedom</t>
+          <t>pressure</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>101165.9293896046</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Supply Gas Specific Heat</t>
+          <t>Manifold Fluid</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>IdealGasSpecificHeats</t>
+          <t>FluidLookup</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>universal_gas_constant</t>
+          <t>temperature</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>8.314</v>
+        <v>300.0153606330658</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Supply Gas Specific Heat</t>
+          <t>Manifold Fluid</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>IdealGasSpecificHeats</t>
+          <t>FluidLookup</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>constant_pressure_specific_heat</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1038.749916111815</v>
+        <v>697.0667889513562</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Supply Gas Specific Heat</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>IdealGasSpecificHeats</t>
+          <t>IsothermalPressureBoundary</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>constant_volume_specific_heat</t>
+          <t>pressure</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>741.9642257941534</v>
+        <v>146271.5950004372</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Supply Gas Specific Heat</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IdealGasSpecificHeats</t>
+          <t>IsothermalPressureBoundary</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>specific_heat_ratio</t>
+          <t>temperature</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1.4</v>
+        <v>299.9964964150044</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Tank Gas</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>GeneralFluidLookupfromPT</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>fluid</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Nitrogen</t>
-        </is>
+          <t>upstream_pressure</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>146271.5950004372</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Tank Gas</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>GeneralFluidLookupfromPT</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>pressure</t>
+          <t>downstream_pressure</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>13789514.586336</v>
+        <v>101165.9293896046</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Tank Gas</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>GeneralFluidLookupfromPT</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>temperature</t>
+          <t>length</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>300</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PR-Reg</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IsentropicGasRegulator</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>upstream_pressure</t>
+          <t>inner_diameter</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>20684271.879504</v>
+        <v>0.0127000254000508</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PR-Reg</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IsentropicGasRegulator</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>upstream_temperature</t>
+          <t>roughness</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>300</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PR-Reg</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>IsentropicGasRegulator</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>set_pressure</t>
+          <t>density</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>13789514.586336</v>
+        <v>697.0951491238991</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PR-Reg</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>IsentropicGasRegulator</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>discharge_coefficient</t>
+          <t>dynamic_viscosity</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>0.0005005309124888494</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PR-Reg</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>IsentropicGasRegulator</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>cross_sectional_area</t>
+          <t>Reynolds_number_threshold</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>3.165316250012662e-05</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PR-Reg</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>IsentropicGasRegulator</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>specific_gas_constant</t>
+          <t>mass_flow</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>296.7856903176614</v>
+        <v>0.6000000000311347</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PR-Reg</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>IsentropicGasRegulator</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>specific_heat_ratio</t>
+          <t>friction_factor</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1.4</v>
+        <v>0.03560027574836816</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PR-Reg</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>IsentropicGasRegulator</t>
+          <t>CircularPipeDarcyWeisbach</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>flow_regime</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>turbulent</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Line 1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>CircularPipeDarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Reynolds_number</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>120178.2498417201</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Manifold</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SimpleVolume</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>pressure</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>101165.9293896046</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Manifold</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>SimpleVolume</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>temperature</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>300.0153606330658</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Manifold</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SimpleVolume</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>density</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>697.0667889513562</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Manifold</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>SimpleVolume</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>volume</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Manifold</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SimpleVolume</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>mass_flow_in</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>0.6000000000311347</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Manifold</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SimpleVolume</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>mass_flow_out</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>0.6000000000528062</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Manifold</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SimpleVolume</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>enthalpy_in</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>-240286.6900943597</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Manifold</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SimpleVolume</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>enthalpy_out</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>-240286.690064993</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>EllipticalDuctDarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>upstream_pressure</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>101165.9293896046</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>EllipticalDuctDarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>downstream_pressure</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>101146.0894907746</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>EllipticalDuctDarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>length</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>EllipticalDuctDarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>semi_major_axis</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>0.05080010160020321</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>EllipticalDuctDarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>semi_minor_axis</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>0.0254000508001016</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>EllipticalDuctDarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>roughness</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>EllipticalDuctDarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>density</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>697.0667889513562</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>EllipticalDuctDarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>dynamic_viscosity</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>0.0005001786116675494</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>EllipticalDuctDarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Reynolds_number_threshold</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>2300</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>EllipticalDuctDarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
           <t>mass_flow</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>1.437245559922177</v>
+      <c r="D40" t="n">
+        <v>0.6000000000528062</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>EllipticalDuctDarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>friction_factor</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>0.02943054453513953</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>EllipticalDuctDarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>flow_regime</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>turbulent</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Line 2</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>EllipticalDuctDarcyWeisbach</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Reynolds_number</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>19498.38013661465</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Atmoshere</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>PressureBoundary</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>pressure</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>101146.0894907746</v>
       </c>
     </row>
   </sheetData>

</xml_diff>